<commit_message>
Late entries and country for new person
</commit_message>
<xml_diff>
--- a/data/2026-03-30/SCW Weekly Comp 2026-03-30 (Responses).xlsx
+++ b/data/2026-03-30/SCW Weekly Comp 2026-03-30 (Responses).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="323">
   <si>
     <t>Timestamp</t>
   </si>
@@ -950,6 +950,36 @@
   </si>
   <si>
     <t>1:04.70</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/events/1215939800337613/?post_id=1220099369921656&amp;view=permalink&amp;__cft__[0]=AZZ61pfk8lE7U4kxphHjrnV3isIYu6lcTlBz1HpR3c7RYgDkxHbqarlgZKTbaB_jXKSo5Ry1caDt3IiM9v5oanU0Y7UsNae1v53FM4XrKncb3eA-xt5uvl_1TU2TPhuC3x8&amp;__tn__=%2CO%2CP-R</t>
+  </si>
+  <si>
+    <t>5:52.69</t>
+  </si>
+  <si>
+    <t>6:53.01</t>
+  </si>
+  <si>
+    <t>6:15.52</t>
+  </si>
+  <si>
+    <t>6:20.41</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/events/1215939800337613/?post_id=1220098243255102&amp;view=permalink&amp;__cft__[0]=AZYTZYxnQmno9TxSspEnm_uzJvmBlMiEoMttJM-O4tZd34j6v5nJSoaj4KcjOLzAEl1FUMDQibm2XADvbKH933iYvmBhvLM5hWLinsqdkwpSLg3gstwuVO6i-Ef-KHPV9eQ&amp;__tn__=%2CO%2CP-R</t>
+  </si>
+  <si>
+    <t>3:42.38</t>
+  </si>
+  <si>
+    <t>3:48.88</t>
+  </si>
+  <si>
+    <t>3:23.27</t>
+  </si>
+  <si>
+    <t>3:38.18</t>
   </si>
 </sst>
 </file>
@@ -1106,7 +1136,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:DH55" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:DH57" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="112">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Name" id="2"/>
@@ -4013,6 +4043,76 @@
         <v>58.57</v>
       </c>
     </row>
+    <row r="56" ht="22.5" customHeight="1">
+      <c r="A56" s="6">
+        <v>46126.96422686343</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="C56" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="D56" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="E56" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="F56" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="AO56" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="AP56" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="AQ56" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="AR56" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="AS56" s="7" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="57" ht="22.5" customHeight="1">
+      <c r="A57" s="6">
+        <v>46126.96477476852</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="D57" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="E57" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="F57" s="8" t="s">
+        <v>318</v>
+      </c>
+      <c r="AJ57" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="AK57" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="AL57" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="AM57" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="AN57" s="7" t="s">
+        <v>322</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="F2"/>
@@ -4069,10 +4169,12 @@
     <hyperlink r:id="rId52" ref="F53"/>
     <hyperlink r:id="rId53" ref="F54"/>
     <hyperlink r:id="rId54" ref="F55"/>
+    <hyperlink r:id="rId55" ref="F56"/>
+    <hyperlink r:id="rId56" ref="F57"/>
   </hyperlinks>
-  <drawing r:id="rId55"/>
+  <drawing r:id="rId57"/>
   <tableParts count="1">
-    <tablePart r:id="rId57"/>
+    <tablePart r:id="rId59"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>